<commit_message>
Implement ad reward system with UIWatchAdsTipsWindow for displaying ad rewards and handling claims. Update GlobalConfig to include AdRewardPackIds and adjust logging levels for error handling in various scripts.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/global_config.xlsx
+++ b/Configs/GameConfig/Datas/global_config.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="31335" windowHeight="15570"/>
+    <workbookView windowWidth="27195" windowHeight="16065"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>##column##var</t>
   </si>
@@ -84,6 +84,18 @@
   </si>
   <si>
     <t>每日签到奖励id</t>
+  </si>
+  <si>
+    <t>ad_reward_pack_ids</t>
+  </si>
+  <si>
+    <t>(list#sep=|),int</t>
+  </si>
+  <si>
+    <t>3001|3002</t>
+  </si>
+  <si>
+    <t>广告礼包ID</t>
   </si>
 </sst>
 </file>
@@ -712,7 +724,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="22" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -720,6 +732,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="22" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1039,8 +1052,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:V8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="7"/>
+  <dimension ref="A1:V9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="25.5" customWidth="1"/>
     <col min="2" max="2" width="17.25" customWidth="1"/>
@@ -1176,6 +1189,20 @@
         <v>18</v>
       </c>
     </row>
+    <row r="9" spans="1:22">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>